<commit_message>
Update BtHoster row: confirmed BTCloud / Limited Network LTD successor + lineage
- Promote to T1-Confirmed BPH (self-advertised bulletproof; both live ASNs on Spamhaus ASN-DROP)
- primary_asn AS214295 -> AS213790 (live); chain AS198465 BtHoster LTD -> Skynet/Inside Network -> Limited Network LTD (AS213790) / AS213388
- Multi-vector attribution: 45.142.193.0/24 inetnum owned by Limited Network LTD, prefix migration (2026-06-23), shared wcd RIPE maintainer; btcloud.ro brand; UK nominee shells; Iranian-prefix false-flag
- Add SECURITYONLINE-BTHOSTER + RIPE-AAWG-BTHOSTER sources (index 50 -> 52)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BPH_Master.xlsx
+++ b/BPH_Master.xlsx
@@ -5269,20 +5269,24 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>T2-High Risk</t>
+          <t>T1-Confirmed BPH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>AS214295</t>
+          <t>AS213790</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>AS215476</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
+          <t>AS213388; AS214295 (dark); AS215476 (dead); AS198465 (predecessor, recycled to CN)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>45.142.193.0/24; 77.90.185.0/24; 172.94.9.0/24; 192.253.248.0/24; 206.123.156.0/24; 185.93.89.0/24; 45.129.14.0/24</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>United Kingdom (shells)</t>
@@ -5290,28 +5294,32 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Lithuania (upstream)</t>
+          <t>Lithuania / Bulgaria (transit)</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Skynet Network Ltd; Inside Network LTD</t>
+          <t>Limited Network LTD; Skynet Network Ltd; Inside Network LTD; BtHoster LTD (predecessor)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>BtHoster</t>
+          <t>BtHoster; BTCloud; btcloud.ro</t>
         </is>
       </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>UAB Host Baltic (AS209605, Lithuania)</t>
+          <t>UAB Host Baltic (AS209605); Tube-Hosting (AS49581, aurologic)</t>
         </is>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Nominee dirs: Murray Charles / Jonathan Reynolds / Brooks William Thomas; provisioned via Khatibi (UAE, wcd maintainer) + Mashayekhi (Iran LIR)</t>
+        </is>
+      </c>
       <c r="P56" t="inlineStr">
         <is>
           <t>Initial Access Brokers</t>
@@ -5324,38 +5332,38 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>AS-leasing; Shell rebranding; Prefix transfer to erase reputation; masscan-server provisioning</t>
+          <t>AS-leasing; Shell rebranding (BtHoster LTD-&gt;Skynet/Inside-&gt;Limited Network); Prefix transfer w/ inetnum retained across ASN rotation; masscan-server provisioning; Iranian-prefix false-flag</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>High malicious traffic ratio; Shell company structure; Prefix churn; Masscan servers (~1300 kpps)</t>
+          <t>On Spamhaus ASN-DROP (AS213790 + AS213388); self-advertised bulletproof (@bthosterltd); masscan ~1300 kpps; shell/nominee structure; shared wcd RIPE maintainer</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr">
         <is>
-          <t>INTRINSEC-BTHOSTER</t>
+          <t>INTRINSEC-BTHOSTER; SECURITYONLINE-BTHOSTER; RIPE-AAWG-BTHOSTER</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>Intrinsec (2025-06-10, high confidence): bulletproof / AS-leasing operator offering pre-configured masscan servers to threat actors via UK shells Skynet Network Ltd (AS214295) and Inside Network LTD (AS215476), upstream UAB Host Baltic (AS209605). Transfers IPv4 prefixes between rebranded entities to erase malicious-activity history.</t>
+          <t>Confirmed multi-vector (2026-06): BtHoster = "BTCloud" operator running recycled UK '[Word] Network LTD' shells -- BtHoster LTD (AS198465, dead 2024-03) -&gt; Skynet Network Ltd (AS214295) + Inside Network LTD (AS215476) (struck off 2025) -&gt; Limited Network LTD (AS213790, ACTIVE) + downstream AS213388. Live identity tied by: the 45.142.193.0/24 inetnum is owned by Limited Network LTD (migrated Skynet-&gt;AS213388 on 2026-06-23, owner unchanged); abuse@btcloud.ro brand on its ARIN blocks; direct AS213790&lt;-&gt;AS214295 peering; shared 'wcd' RIPE maintainer (Khatibi/UAE). Sells pre-configured masscan servers (~1300 kpps) to Initial Access Brokers; transfers prefixes between shells to erase reputation; reuses Iranian-origin prefixes to fake Iran attribution. Both live ASNs on Spamhaus ASN-DROP. Transit via UAB Host Baltic (AS209605) + Tube-Hosting (AS49581, aurologic) with a Bulgarian backstop (SS-NET AS204428 / 4Vendeta). Full attribution dossier in internal investigation.</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>UK-shell AS-leasing bulletproof operator using prefix-transfer rebrands to erase reputation; provisions masscan/scanning servers.</t>
+          <t>Confirmed bulletproof / AS-leasing operator ('BTCloud') running rotating UK nominee shells; live as Limited Network LTD (AS213790)/AS213388; masscan-as-a-service to IABs.</t>
         </is>
       </c>
     </row>

</xml_diff>